<commit_message>
Enhance working budget functionality: add image handling for Excel export, improve data formatting, and update PDF layout
</commit_message>
<xml_diff>
--- a/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
+++ b/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SCV\NAKANO\HOAN_NAKANO\src\FileCabinet\SuiteScripts\Nkn\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{645476A2-0D30-408C-8EE8-3CF36E19230F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19EC08B-1840-470E-AF5B-8AA4254D3CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FBFDA3B2-B482-4DA1-B36E-083EA194CE53}"/>
+    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" xr2:uid="{FBFDA3B2-B482-4DA1-B36E-083EA194CE53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -252,12 +252,6 @@
     <t>{pConsultantQS}</t>
   </si>
   <si>
-    <t>{pConstructionPeriodStart} ~ {pConstructionPeriodEnd}</t>
-  </si>
-  <si>
-    <t>{pdefectsLiabilityPeriod}</t>
-  </si>
-  <si>
     <t>{pTypeOfContract}</t>
   </si>
   <si>
@@ -300,9 +294,6 @@
     <t>{pSteelStructure}</t>
   </si>
   <si>
-    <t>{pPrimaryCurrency</t>
-  </si>
-  <si>
     <t>{pContractSum}</t>
   </si>
   <si>
@@ -312,33 +303,18 @@
     <t>{pTotalProfit}</t>
   </si>
   <si>
-    <t>{pTotalProfitPer}</t>
-  </si>
-  <si>
     <t>{pOverhead}</t>
   </si>
   <si>
-    <t>{pOverheadPer}</t>
-  </si>
-  <si>
     <t>{pProfitAttendance}</t>
   </si>
   <si>
-    <t>{pProfitAttendancePer}</t>
-  </si>
-  <si>
     <t>{pAwardProfit}</t>
   </si>
   <si>
-    <t>{pAwardProfitPer}</t>
-  </si>
-  <si>
     <t>{pPcSumProvSum}</t>
   </si>
   <si>
-    <t>{pPcSumProvSumPer}</t>
-  </si>
-  <si>
     <t>{pContractSumByGFA}</t>
   </si>
   <si>
@@ -360,7 +336,31 @@
     <t>{pIndirectExpenses}</t>
   </si>
   <si>
-    <t>{pIndirectExpensesPer}</t>
+    <t>{pPrimaryCurrency}</t>
+  </si>
+  <si>
+    <t>{pDefectsLiabilityPeriod}</t>
+  </si>
+  <si>
+    <t>{pConstructionPeriodStart} ~ {pConstructionPeriodEnd} ({pConstructionPeriodMonths})</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{pTotalProfitPer}% </t>
+  </si>
+  <si>
+    <t>{pOverheadPer}%</t>
+  </si>
+  <si>
+    <t>{pProfitAttendancePer}%</t>
+  </si>
+  <si>
+    <t>{pAwardProfitPer}%</t>
+  </si>
+  <si>
+    <t>{pPcSumProvSumPer}%</t>
+  </si>
+  <si>
+    <t>{pIndirectExpensesPer}%</t>
   </si>
   <si>
     <t>{pImage}</t>
@@ -414,7 +414,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -554,8 +554,152 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF000000"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="dotted">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
@@ -567,9 +711,22 @@
     <border>
       <left/>
       <right/>
-      <top/>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
       <bottom style="double">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -577,65 +734,34 @@
       <left/>
       <right style="medium">
         <color rgb="FF000000"/>
+      </right>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="double">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="double">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="double">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="dotted">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="dotted">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="double">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="dotted">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="dotted">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="double">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="dotted">
-        <color rgb="FF000000"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -643,7 +769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -669,12 +795,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -684,31 +804,156 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -717,101 +962,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1127,45 +1309,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{573A7AD8-49DB-4C7D-B078-908BDA7FB167}">
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="4" max="4" width="5.77734375" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.109375" customWidth="1"/>
     <col min="12" max="12" width="13.33203125" customWidth="1"/>
     <col min="15" max="15" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.88671875" customWidth="1"/>
+    <col min="18" max="18" width="5.44140625" customWidth="1"/>
+    <col min="19" max="19" width="6.5546875" customWidth="1"/>
+    <col min="20" max="20" width="6.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="25.2" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="38"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="19"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
@@ -1186,7 +1372,7 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
-      <c r="S2" s="39"/>
+      <c r="S2" s="18"/>
     </row>
     <row r="3" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -1196,34 +1382,34 @@
       <c r="C3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="51" t="s">
+      <c r="D3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="12">
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="10">
         <v>1</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="11" t="s">
         <v>35</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="11" t="s">
+      <c r="M3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="R3" s="25"/>
-      <c r="S3" s="40"/>
+      <c r="N3" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O3" s="2"/>
+      <c r="P3" s="64" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="20"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
@@ -1244,7 +1430,7 @@
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
-      <c r="S4" s="39"/>
+      <c r="S4" s="18"/>
     </row>
     <row r="5" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -1254,17 +1440,17 @@
       <c r="C5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="12">
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="10">
         <v>2</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="J5" s="11" t="s">
         <v>37</v>
       </c>
       <c r="K5" s="2"/>
@@ -1272,26 +1458,26 @@
       <c r="M5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="N5" s="2"/>
-      <c r="O5" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="R5" s="26"/>
-      <c r="S5" s="40"/>
+      <c r="N5" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O5" s="2"/>
+      <c r="P5" s="68" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="23"/>
+      <c r="S5" s="20"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -1302,40 +1488,40 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-      <c r="S6" s="39"/>
+      <c r="S6" s="18"/>
     </row>
     <row r="7" spans="1:19" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="12">
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="10">
         <v>3</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="11" t="s">
         <v>38</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="M7" s="11" t="s">
+      <c r="M7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="11" t="s">
+      <c r="N7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O7" s="2"/>
+      <c r="P7" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="R7" s="25"/>
-      <c r="S7" s="14" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q7" s="64"/>
+      <c r="R7" s="69" t="s">
+        <v>103</v>
+      </c>
+      <c r="S7" s="70"/>
     </row>
     <row r="8" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
@@ -1355,18 +1541,18 @@
       <c r="M8" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="N8" s="2"/>
-      <c r="O8" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="R8" s="28"/>
-      <c r="S8" s="15" t="s">
-        <v>94</v>
-      </c>
+      <c r="N8" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O8" s="2"/>
+      <c r="P8" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q8" s="65"/>
+      <c r="R8" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="S8" s="72"/>
     </row>
     <row r="9" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
@@ -1386,18 +1572,18 @@
       <c r="M9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="N9" s="2"/>
-      <c r="O9" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="R9" s="29"/>
-      <c r="S9" s="15" t="s">
-        <v>96</v>
-      </c>
+      <c r="N9" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O9" s="2"/>
+      <c r="P9" s="55" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q9" s="55"/>
+      <c r="R9" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="S9" s="59"/>
     </row>
     <row r="10" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1407,13 +1593,13 @@
       <c r="C10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="51" t="s">
+      <c r="D10" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="51"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -1421,21 +1607,21 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="41"/>
-      <c r="R10" s="41"/>
-      <c r="S10" s="39"/>
+      <c r="P10" s="56"/>
+      <c r="Q10" s="56"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="18"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="12">
+      <c r="D11" s="2"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="10">
         <v>4</v>
       </c>
       <c r="J11" s="6" t="s">
@@ -1448,10 +1634,10 @@
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="42"/>
-      <c r="R11" s="42"/>
-      <c r="S11" s="43"/>
+      <c r="P11" s="47"/>
+      <c r="Q11" s="47"/>
+      <c r="R11" s="47"/>
+      <c r="S11" s="50"/>
     </row>
     <row r="12" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
@@ -1469,18 +1655,18 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="R12" s="27"/>
-      <c r="S12" s="15" t="s">
-        <v>98</v>
-      </c>
+      <c r="N12" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O12" s="2"/>
+      <c r="P12" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q12" s="55"/>
+      <c r="R12" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="S12" s="59"/>
     </row>
     <row r="13" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
@@ -1498,18 +1684,18 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="R13" s="29"/>
-      <c r="S13" s="16" t="s">
+      <c r="N13" s="9" t="s">
         <v>100</v>
       </c>
+      <c r="O13" s="2"/>
+      <c r="P13" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q13" s="62"/>
+      <c r="R13" s="73" t="s">
+        <v>107</v>
+      </c>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="1:19" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
@@ -1530,7 +1716,7 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
-      <c r="S14" s="39"/>
+      <c r="S14" s="18"/>
     </row>
     <row r="15" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -1540,14 +1726,14 @@
       <c r="C15" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="D15" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
-      <c r="G15" s="51"/>
-      <c r="H15" s="51"/>
-      <c r="I15" s="12">
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="48"/>
+      <c r="I15" s="10">
         <v>5</v>
       </c>
       <c r="J15" s="2" t="s">
@@ -1561,7 +1747,7 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
-      <c r="S15" s="39"/>
+      <c r="S15" s="18"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
@@ -1584,7 +1770,7 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
-      <c r="S16" s="39"/>
+      <c r="S16" s="18"/>
     </row>
     <row r="17" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -1594,13 +1780,13 @@
       <c r="C17" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="51" t="s">
+      <c r="D17" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="E17" s="51"/>
-      <c r="F17" s="51"/>
-      <c r="G17" s="51"/>
-      <c r="H17" s="55" t="s">
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="27" t="s">
         <v>12</v>
       </c>
       <c r="I17" s="2"/>
@@ -1610,20 +1796,20 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="N17" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="Q17" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="R17" s="31"/>
-      <c r="S17" s="17" t="s">
+      <c r="P17" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q17" s="63"/>
+      <c r="R17" s="75" t="s">
         <v>49</v>
       </c>
+      <c r="S17" s="76"/>
     </row>
     <row r="18" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
@@ -1641,32 +1827,32 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="N18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="Q18" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="R18" s="10"/>
-      <c r="S18" s="17" t="s">
+      <c r="P18" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q18" s="53"/>
+      <c r="R18" s="77" t="s">
         <v>49</v>
       </c>
+      <c r="S18" s="78"/>
     </row>
     <row r="19" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="51" t="s">
+      <c r="D19" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="51"/>
-      <c r="F19" s="51"/>
-      <c r="G19" s="51"/>
-      <c r="H19" s="55" t="s">
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="27" t="s">
         <v>13</v>
       </c>
       <c r="I19" s="2"/>
@@ -1681,7 +1867,7 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
-      <c r="S19" s="39"/>
+      <c r="S19" s="18"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
@@ -1699,32 +1885,32 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="11" t="s">
+      <c r="N20" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="P20" s="2" t="s">
+      <c r="O20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="Q20" s="32" t="s">
-        <v>103</v>
-      </c>
-      <c r="R20" s="32"/>
-      <c r="S20" s="17" t="s">
+      <c r="P20" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q20" s="58"/>
+      <c r="R20" s="75" t="s">
         <v>49</v>
       </c>
+      <c r="S20" s="76"/>
     </row>
     <row r="21" spans="1:19" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="51" t="s">
+      <c r="D21" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
-      <c r="G21" s="51"/>
-      <c r="H21" s="55" t="s">
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="27" t="s">
         <v>14</v>
       </c>
       <c r="I21" s="2"/>
@@ -1737,7 +1923,7 @@
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
-      <c r="S21" s="39"/>
+      <c r="S21" s="18"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
@@ -1748,7 +1934,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="12">
+      <c r="I22" s="10">
         <v>6</v>
       </c>
       <c r="J22" s="6" t="s">
@@ -1764,19 +1950,19 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
-      <c r="S22" s="39"/>
+      <c r="S22" s="18"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="51" t="s">
+      <c r="D23" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="56" t="s">
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="28" t="s">
         <v>15</v>
       </c>
       <c r="I23" s="2"/>
@@ -1790,12 +1976,12 @@
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="R23" s="30"/>
-      <c r="S23" s="44"/>
+      <c r="P23" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q23" s="60"/>
+      <c r="R23" s="60"/>
+      <c r="S23" s="61"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
@@ -1817,24 +2003,24 @@
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="R24" s="10"/>
-      <c r="S24" s="33"/>
+      <c r="P24" s="53" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q24" s="53"/>
+      <c r="R24" s="53"/>
+      <c r="S24" s="54"/>
     </row>
     <row r="25" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="51" t="s">
+      <c r="D25" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="55" t="s">
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="27" t="s">
         <v>16</v>
       </c>
       <c r="I25" s="2"/>
@@ -1848,12 +2034,12 @@
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="R25" s="10"/>
-      <c r="S25" s="33"/>
+      <c r="P25" s="53" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q25" s="53"/>
+      <c r="R25" s="53"/>
+      <c r="S25" s="54"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
@@ -1874,22 +2060,22 @@
       <c r="P26" s="2"/>
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
-      <c r="S26" s="39"/>
+      <c r="S26" s="18"/>
     </row>
     <row r="27" spans="1:19" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="51" t="s">
+      <c r="D27" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="55" t="s">
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="12">
+      <c r="I27" s="10">
         <v>7</v>
       </c>
       <c r="J27" s="2" t="s">
@@ -1903,7 +2089,7 @@
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
-      <c r="S27" s="39"/>
+      <c r="S27" s="18"/>
     </row>
     <row r="28" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
@@ -1915,7 +2101,7 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="12" t="s">
+      <c r="J28" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K28" s="6" t="s">
@@ -1923,34 +2109,34 @@
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="R28" s="27"/>
-      <c r="S28" s="15" t="s">
+      <c r="N28" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="O28" s="2"/>
+      <c r="P28" s="55" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q28" s="55"/>
+      <c r="R28" s="58" t="s">
         <v>108</v>
       </c>
+      <c r="S28" s="59"/>
     </row>
     <row r="29" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E29" s="51" t="s">
-        <v>72</v>
-      </c>
+      <c r="D29" s="51" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="51"/>
       <c r="F29" s="51"/>
       <c r="G29" s="51"/>
-      <c r="H29" s="51"/>
+      <c r="H29" s="27"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
@@ -1958,28 +2144,28 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="41"/>
-      <c r="R29" s="41"/>
-      <c r="S29" s="45"/>
+      <c r="P29" s="56"/>
+      <c r="Q29" s="56"/>
+      <c r="R29" s="56"/>
+      <c r="S29" s="57"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E30" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="55" t="s">
+      <c r="D30" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="29" t="s">
         <v>58</v>
       </c>
+      <c r="H30" s="29"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
@@ -1987,20 +2173,28 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="42"/>
-      <c r="R30" s="42"/>
-      <c r="S30" s="43"/>
+      <c r="P30" s="47"/>
+      <c r="Q30" s="47"/>
+      <c r="R30" s="47"/>
+      <c r="S30" s="50"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
+      <c r="A31" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
-      <c r="G31" s="55"/>
-      <c r="H31" s="55"/>
+      <c r="C31" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D31" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="51"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="H31" s="27"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
@@ -2009,27 +2203,25 @@
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
-      <c r="Q31" s="42"/>
-      <c r="R31" s="42"/>
-      <c r="S31" s="43"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
+      <c r="S31" s="18"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E32" s="50" t="s">
-        <v>74</v>
-      </c>
-      <c r="F32" s="50"/>
-      <c r="G32" s="50"/>
-      <c r="H32" s="55" t="s">
-        <v>60</v>
-      </c>
+      <c r="D32" s="52" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="52"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="52"/>
+      <c r="H32" s="25"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
@@ -2040,17 +2232,25 @@
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
-      <c r="S32" s="39"/>
+      <c r="S32" s="18"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A33" s="3"/>
+      <c r="A33" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
+      <c r="C33" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" s="52"/>
+      <c r="F33" s="52"/>
+      <c r="G33" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="H33" s="25"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -2061,23 +2261,17 @@
       <c r="P33" s="2"/>
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
-      <c r="S33" s="39"/>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E34" s="50" t="s">
-        <v>75</v>
-      </c>
-      <c r="F34" s="50"/>
-      <c r="G34" s="50"/>
-      <c r="H34" s="50"/>
+      <c r="S33" s="18"/>
+    </row>
+    <row r="34" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="14"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
@@ -2088,17 +2282,19 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
-      <c r="S34" s="39"/>
+      <c r="S34" s="18"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
+      <c r="A35" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="30"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -2109,25 +2305,23 @@
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
       <c r="R35" s="2"/>
-      <c r="S35" s="39"/>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>19</v>
+      <c r="S35" s="18"/>
+    </row>
+    <row r="36" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E36" s="50" t="s">
-        <v>76</v>
-      </c>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="55" t="s">
-        <v>62</v>
-      </c>
+      <c r="D36" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="43"/>
+      <c r="H36" s="4"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
@@ -2136,19 +2330,25 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="2"/>
-      <c r="S36" s="39"/>
-    </row>
-    <row r="37" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="46"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="47"/>
-      <c r="E37" s="47"/>
-      <c r="F37" s="47"/>
-      <c r="G37" s="47"/>
-      <c r="H37" s="47"/>
+      <c r="Q36" s="47"/>
+      <c r="R36" s="47"/>
+      <c r="S36" s="18"/>
+    </row>
+    <row r="37" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="E37" s="44"/>
+      <c r="F37" s="44"/>
+      <c r="G37" s="44"/>
+      <c r="H37" s="4"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
@@ -2159,19 +2359,25 @@
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
       <c r="R37" s="2"/>
-      <c r="S37" s="39"/>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S37" s="18"/>
+    </row>
+    <row r="38" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="4"/>
+      <c r="C38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38" s="44" t="s">
+        <v>77</v>
+      </c>
+      <c r="E38" s="44"/>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
@@ -2182,23 +2388,25 @@
       <c r="P38" s="2"/>
       <c r="Q38" s="2"/>
       <c r="R38" s="2"/>
-      <c r="S38" s="39"/>
-    </row>
-    <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>21</v>
+      <c r="S38" s="18"/>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E39" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="F39" s="34"/>
-      <c r="G39" s="34"/>
-      <c r="H39" s="4"/>
+      <c r="D39" s="45" t="s">
+        <v>78</v>
+      </c>
+      <c r="E39" s="45"/>
+      <c r="F39" s="45"/>
+      <c r="G39" s="45"/>
+      <c r="H39" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
@@ -2207,25 +2415,27 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
-      <c r="Q39" s="42"/>
-      <c r="R39" s="42"/>
-      <c r="S39" s="39"/>
+      <c r="Q39" s="2"/>
+      <c r="R39" s="2"/>
+      <c r="S39" s="18"/>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E40" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="4"/>
+      <c r="D40" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="46"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="46"/>
+      <c r="H40" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
@@ -2236,25 +2446,17 @@
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
-      <c r="S40" s="39"/>
+      <c r="S40" s="18"/>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A41" s="3"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
-      <c r="D41" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="4"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
@@ -2265,25 +2467,17 @@
       <c r="P41" s="2"/>
       <c r="Q41" s="2"/>
       <c r="R41" s="2"/>
-      <c r="S41" s="39"/>
+      <c r="S41" s="18"/>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="A42" s="3"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="4"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
@@ -2294,24 +2488,28 @@
       <c r="P42" s="2"/>
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
-      <c r="S42" s="39"/>
+      <c r="S42" s="18"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E43" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43" s="10"/>
+      <c r="E43" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="F43" s="2"/>
+      <c r="G43" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="4" t="s">
-        <v>24</v>
+      <c r="H43" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -2323,17 +2521,29 @@
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
-      <c r="S43" s="39"/>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A44" s="3"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="S43" s="18"/>
+    </row>
+    <row r="44" spans="1:19" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C44" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="D44" s="10"/>
+      <c r="E44" s="26" t="s">
+        <v>33</v>
+      </c>
       <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="4"/>
+      <c r="G44" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="H44" s="40" t="s">
+        <v>30</v>
+      </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -2344,83 +2554,62 @@
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
-      <c r="S44" s="39"/>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A45" s="3"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
+      <c r="S44" s="18"/>
+    </row>
+    <row r="45" spans="1:19" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D45" s="10"/>
+      <c r="E45" s="26" t="s">
+        <v>65</v>
+      </c>
       <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="39"/>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D46" s="2"/>
-      <c r="E46" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F46" s="2"/>
-      <c r="G46" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
-      <c r="S46" s="39"/>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D47" s="2"/>
-      <c r="E47" s="6" t="s">
-        <v>33</v>
-      </c>
+      <c r="G45" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I45" s="34"/>
+      <c r="S45" s="42"/>
+    </row>
+    <row r="46" spans="1:19" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="33"/>
+      <c r="B46" s="38"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="41"/>
+      <c r="I46" s="35"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="16"/>
+      <c r="L46" s="16"/>
+      <c r="M46" s="16"/>
+      <c r="N46" s="16"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="16"/>
+      <c r="R46" s="16"/>
+      <c r="S46" s="21"/>
+    </row>
+    <row r="47" spans="1:19" ht="16.8" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="2"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="26"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="H47" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="G47" s="2"/>
+      <c r="H47" s="10"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
@@ -2431,87 +2620,61 @@
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
-      <c r="S47" s="39"/>
-    </row>
-    <row r="48" spans="1:19" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" s="48"/>
-      <c r="E48" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="F48" s="48"/>
-      <c r="G48" s="48" t="s">
-        <v>87</v>
-      </c>
-      <c r="H48" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="I48" s="48"/>
-      <c r="J48" s="48"/>
-      <c r="K48" s="48"/>
-      <c r="L48" s="48"/>
-      <c r="M48" s="48"/>
-      <c r="N48" s="48"/>
-      <c r="O48" s="48"/>
-      <c r="P48" s="48"/>
-      <c r="Q48" s="48"/>
-      <c r="R48" s="48"/>
-      <c r="S48" s="49"/>
-    </row>
-    <row r="49" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="S47" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="Q39:R39"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="E43:G43"/>
+  <mergeCells count="51">
+    <mergeCell ref="R12:S12"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="Q36:R36"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="D5:H5"/>
     <mergeCell ref="D15:H15"/>
     <mergeCell ref="D17:G17"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="Q30:S30"/>
-    <mergeCell ref="Q31:S31"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="E34:H34"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="Q24:S24"/>
-    <mergeCell ref="Q25:S25"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="Q29:S29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="E29:H29"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q23:S23"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D30:F30"/>
     <mergeCell ref="E11:H11"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="P30:S30"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="D32:G32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="P24:S24"/>
+    <mergeCell ref="P25:S25"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="P29:S29"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="D39:G39"/>
+    <mergeCell ref="D40:G40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor scv_print_po_my.js, scv_print_rpo_my.js, scv_print_wb.js, and XML files: update labels, improve formatting, and enhance readability
</commit_message>
<xml_diff>
--- a/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
+++ b/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SCV\NAKANO\HOAN_NAKANO\src\FileCabinet\SuiteScripts\Nkn\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD39AAA8-5DCF-4C4A-9AA1-49858329B1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548FF733-0829-4D61-A634-96E9730F7893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FBFDA3B2-B482-4DA1-B36E-083EA194CE53}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="111">
   <si>
     <t>WORKING BUDGET</t>
   </si>
@@ -364,6 +364,9 @@
   </si>
   <si>
     <t>{pIndirectExpensesPer}%</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NAKANO SINGAPORE </t>
   </si>
 </sst>
 </file>
@@ -879,14 +882,107 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -896,103 +992,10 @@
     <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1312,7 +1315,7 @@
   <dimension ref="A1:S47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" customWidth="1"/>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
     <col min="4" max="4" width="5.77734375" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
@@ -1328,23 +1331,25 @@
     <col min="20" max="20" width="6.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="25.2" thickTop="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:19" ht="69.599999999999994" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="A1" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
+      <c r="B1" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
       <c r="F1" s="13"/>
-      <c r="G1" s="67" t="s">
+      <c r="G1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
       <c r="M1" s="13"/>
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
@@ -1382,13 +1387,13 @@
       <c r="C3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
       <c r="I3" s="10">
         <v>1</v>
       </c>
@@ -1404,10 +1409,10 @@
         <v>101</v>
       </c>
       <c r="O3" s="2"/>
-      <c r="P3" s="64" t="s">
+      <c r="P3" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="Q3" s="64"/>
+      <c r="Q3" s="51"/>
       <c r="R3" s="22"/>
       <c r="S3" s="20"/>
     </row>
@@ -1440,13 +1445,13 @@
       <c r="C5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="D5" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
       <c r="I5" s="10">
         <v>2</v>
       </c>
@@ -1462,10 +1467,10 @@
         <v>101</v>
       </c>
       <c r="O5" s="2"/>
-      <c r="P5" s="68" t="s">
+      <c r="P5" s="52" t="s">
         <v>87</v>
       </c>
-      <c r="Q5" s="68"/>
+      <c r="Q5" s="52"/>
       <c r="R5" s="23"/>
       <c r="S5" s="20"/>
     </row>
@@ -1514,14 +1519,14 @@
         <v>101</v>
       </c>
       <c r="O7" s="2"/>
-      <c r="P7" s="64" t="s">
+      <c r="P7" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="Q7" s="64"/>
-      <c r="R7" s="69" t="s">
+      <c r="Q7" s="51"/>
+      <c r="R7" s="55" t="s">
         <v>104</v>
       </c>
-      <c r="S7" s="70"/>
+      <c r="S7" s="56"/>
     </row>
     <row r="8" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
@@ -1545,14 +1550,14 @@
         <v>101</v>
       </c>
       <c r="O8" s="2"/>
-      <c r="P8" s="65" t="s">
+      <c r="P8" s="62" t="s">
         <v>89</v>
       </c>
-      <c r="Q8" s="65"/>
-      <c r="R8" s="71" t="s">
+      <c r="Q8" s="62"/>
+      <c r="R8" s="57" t="s">
         <v>105</v>
       </c>
-      <c r="S8" s="72"/>
+      <c r="S8" s="58"/>
     </row>
     <row r="9" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
@@ -1576,14 +1581,14 @@
         <v>101</v>
       </c>
       <c r="O9" s="2"/>
-      <c r="P9" s="55" t="s">
+      <c r="P9" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="Q9" s="55"/>
-      <c r="R9" s="58" t="s">
+      <c r="Q9" s="59"/>
+      <c r="R9" s="42" t="s">
         <v>106</v>
       </c>
-      <c r="S9" s="59"/>
+      <c r="S9" s="43"/>
     </row>
     <row r="10" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1593,13 +1598,13 @@
       <c r="C10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="48" t="s">
+      <c r="D10" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -1607,8 +1612,8 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="56"/>
+      <c r="P10" s="63"/>
+      <c r="Q10" s="63"/>
       <c r="R10" s="2"/>
       <c r="S10" s="18"/>
     </row>
@@ -1617,10 +1622,10 @@
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
+      <c r="E11" s="53"/>
+      <c r="F11" s="53"/>
+      <c r="G11" s="53"/>
+      <c r="H11" s="53"/>
       <c r="I11" s="10">
         <v>4</v>
       </c>
@@ -1634,10 +1639,10 @@
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="47"/>
-      <c r="Q11" s="47"/>
-      <c r="R11" s="47"/>
-      <c r="S11" s="50"/>
+      <c r="P11" s="53"/>
+      <c r="Q11" s="53"/>
+      <c r="R11" s="53"/>
+      <c r="S11" s="54"/>
     </row>
     <row r="12" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
@@ -1659,14 +1664,14 @@
         <v>101</v>
       </c>
       <c r="O12" s="2"/>
-      <c r="P12" s="55" t="s">
+      <c r="P12" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="Q12" s="55"/>
-      <c r="R12" s="58" t="s">
+      <c r="Q12" s="59"/>
+      <c r="R12" s="42" t="s">
         <v>107</v>
       </c>
-      <c r="S12" s="59"/>
+      <c r="S12" s="43"/>
     </row>
     <row r="13" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
@@ -1688,14 +1693,14 @@
         <v>101</v>
       </c>
       <c r="O13" s="2"/>
-      <c r="P13" s="62" t="s">
+      <c r="P13" s="60" t="s">
         <v>92</v>
       </c>
-      <c r="Q13" s="62"/>
-      <c r="R13" s="73" t="s">
+      <c r="Q13" s="60"/>
+      <c r="R13" s="44" t="s">
         <v>108</v>
       </c>
-      <c r="S13" s="74"/>
+      <c r="S13" s="45"/>
     </row>
     <row r="14" spans="1:19" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
@@ -1726,13 +1731,13 @@
       <c r="C15" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="48"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
       <c r="I15" s="10">
         <v>5</v>
       </c>
@@ -1780,12 +1785,12 @@
       <c r="C17" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="48" t="s">
+      <c r="D17" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="48"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="64"/>
       <c r="H17" s="27" t="s">
         <v>12</v>
       </c>
@@ -1802,14 +1807,14 @@
       <c r="O17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P17" s="63" t="s">
+      <c r="P17" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="Q17" s="63"/>
-      <c r="R17" s="75" t="s">
+      <c r="Q17" s="61"/>
+      <c r="R17" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="S17" s="76"/>
+      <c r="S17" s="47"/>
     </row>
     <row r="18" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
@@ -1833,25 +1838,25 @@
       <c r="O18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P18" s="53" t="s">
+      <c r="P18" s="66" t="s">
         <v>94</v>
       </c>
-      <c r="Q18" s="53"/>
-      <c r="R18" s="77" t="s">
+      <c r="Q18" s="66"/>
+      <c r="R18" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="S18" s="78"/>
+      <c r="S18" s="49"/>
     </row>
     <row r="19" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="48" t="s">
+      <c r="D19" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
+      <c r="E19" s="64"/>
+      <c r="F19" s="64"/>
+      <c r="G19" s="64"/>
       <c r="H19" s="27" t="s">
         <v>13</v>
       </c>
@@ -1891,25 +1896,25 @@
       <c r="O20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P20" s="58" t="s">
+      <c r="P20" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="Q20" s="58"/>
-      <c r="R20" s="75" t="s">
+      <c r="Q20" s="42"/>
+      <c r="R20" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="S20" s="76"/>
+      <c r="S20" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="48" t="s">
+      <c r="D21" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48"/>
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
       <c r="H21" s="27" t="s">
         <v>14</v>
       </c>
@@ -1956,12 +1961,12 @@
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="64" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
+      <c r="E23" s="64"/>
+      <c r="F23" s="64"/>
+      <c r="G23" s="64"/>
       <c r="H23" s="28" t="s">
         <v>15</v>
       </c>
@@ -1976,12 +1981,12 @@
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="60" t="s">
+      <c r="P23" s="67" t="s">
         <v>96</v>
       </c>
-      <c r="Q23" s="60"/>
-      <c r="R23" s="60"/>
-      <c r="S23" s="61"/>
+      <c r="Q23" s="67"/>
+      <c r="R23" s="67"/>
+      <c r="S23" s="68"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
@@ -2003,23 +2008,23 @@
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="53" t="s">
+      <c r="P24" s="66" t="s">
         <v>97</v>
       </c>
-      <c r="Q24" s="53"/>
-      <c r="R24" s="53"/>
-      <c r="S24" s="54"/>
+      <c r="Q24" s="66"/>
+      <c r="R24" s="66"/>
+      <c r="S24" s="72"/>
     </row>
     <row r="25" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
+      <c r="E25" s="64"/>
+      <c r="F25" s="64"/>
+      <c r="G25" s="64"/>
       <c r="H25" s="27" t="s">
         <v>16</v>
       </c>
@@ -2034,12 +2039,12 @@
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="53" t="s">
+      <c r="P25" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="Q25" s="53"/>
-      <c r="R25" s="53"/>
-      <c r="S25" s="54"/>
+      <c r="Q25" s="66"/>
+      <c r="R25" s="66"/>
+      <c r="S25" s="72"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
@@ -2066,12 +2071,12 @@
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="48" t="s">
+      <c r="D27" s="64" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
+      <c r="E27" s="64"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
       <c r="H27" s="27" t="s">
         <v>17</v>
       </c>
@@ -2113,14 +2118,14 @@
         <v>101</v>
       </c>
       <c r="O28" s="2"/>
-      <c r="P28" s="55" t="s">
+      <c r="P28" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="Q28" s="55"/>
-      <c r="R28" s="58" t="s">
+      <c r="Q28" s="59"/>
+      <c r="R28" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="S28" s="59"/>
+      <c r="S28" s="43"/>
     </row>
     <row r="29" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2130,12 +2135,12 @@
       <c r="C29" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="65" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="51"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="51"/>
+      <c r="E29" s="65"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
       <c r="H29" s="27"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -2144,10 +2149,10 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="56"/>
-      <c r="Q29" s="56"/>
-      <c r="R29" s="56"/>
-      <c r="S29" s="57"/>
+      <c r="P29" s="63"/>
+      <c r="Q29" s="63"/>
+      <c r="R29" s="63"/>
+      <c r="S29" s="73"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -2157,11 +2162,11 @@
       <c r="C30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D30" s="46" t="s">
+      <c r="D30" s="70" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
+      <c r="E30" s="70"/>
+      <c r="F30" s="70"/>
       <c r="G30" s="29" t="s">
         <v>58</v>
       </c>
@@ -2173,10 +2178,10 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="47"/>
-      <c r="Q30" s="47"/>
-      <c r="R30" s="47"/>
-      <c r="S30" s="50"/>
+      <c r="P30" s="53"/>
+      <c r="Q30" s="53"/>
+      <c r="R30" s="53"/>
+      <c r="S30" s="54"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -2186,11 +2191,11 @@
       <c r="C31" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D31" s="51" t="s">
+      <c r="D31" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="51"/>
-      <c r="F31" s="51"/>
+      <c r="E31" s="65"/>
+      <c r="F31" s="65"/>
       <c r="G31" s="27" t="s">
         <v>60</v>
       </c>
@@ -2215,12 +2220,12 @@
       <c r="C32" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D32" s="52" t="s">
+      <c r="D32" s="71" t="s">
         <v>73</v>
       </c>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
+      <c r="E32" s="71"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="71"/>
       <c r="H32" s="25"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -2242,11 +2247,11 @@
       <c r="C33" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D33" s="52" t="s">
+      <c r="D33" s="71" t="s">
         <v>74</v>
       </c>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
+      <c r="E33" s="71"/>
+      <c r="F33" s="71"/>
       <c r="G33" s="25" t="s">
         <v>62</v>
       </c>
@@ -2315,12 +2320,12 @@
       <c r="C36" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D36" s="43" t="s">
+      <c r="D36" s="74" t="s">
         <v>75</v>
       </c>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
+      <c r="E36" s="74"/>
+      <c r="F36" s="74"/>
+      <c r="G36" s="74"/>
       <c r="H36" s="4"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -2330,8 +2335,8 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="47"/>
-      <c r="R36" s="47"/>
+      <c r="Q36" s="53"/>
+      <c r="R36" s="53"/>
       <c r="S36" s="18"/>
     </row>
     <row r="37" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2342,12 +2347,12 @@
       <c r="C37" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D37" s="44" t="s">
+      <c r="D37" s="75" t="s">
         <v>76</v>
       </c>
-      <c r="E37" s="44"/>
-      <c r="F37" s="44"/>
-      <c r="G37" s="44"/>
+      <c r="E37" s="75"/>
+      <c r="F37" s="75"/>
+      <c r="G37" s="75"/>
       <c r="H37" s="4"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -2369,12 +2374,12 @@
       <c r="C38" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D38" s="44" t="s">
+      <c r="D38" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="E38" s="44"/>
-      <c r="F38" s="44"/>
-      <c r="G38" s="44"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
       <c r="H38" s="4" t="s">
         <v>24</v>
       </c>
@@ -2398,12 +2403,12 @@
       <c r="C39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D39" s="45" t="s">
+      <c r="D39" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
       <c r="H39" s="4" t="s">
         <v>24</v>
       </c>
@@ -2427,12 +2432,12 @@
       <c r="C40" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D40" s="46" t="s">
+      <c r="D40" s="70" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="46"/>
-      <c r="F40" s="46"/>
-      <c r="G40" s="46"/>
+      <c r="E40" s="70"/>
+      <c r="F40" s="70"/>
+      <c r="G40" s="70"/>
       <c r="H40" s="4" t="s">
         <v>24</v>
       </c>
@@ -2541,7 +2546,7 @@
       <c r="G44" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="H44" s="40" t="s">
+      <c r="H44" s="39" t="s">
         <v>30</v>
       </c>
       <c r="I44" s="2"/>
@@ -2571,14 +2576,14 @@
         <v>65</v>
       </c>
       <c r="F45" s="2"/>
-      <c r="G45" s="39" t="s">
+      <c r="G45" s="77" t="s">
         <v>85</v>
       </c>
       <c r="H45" s="10" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="34"/>
-      <c r="S45" s="42"/>
+      <c r="S45" s="41"/>
     </row>
     <row r="46" spans="1:19" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="33"/>
@@ -2588,7 +2593,7 @@
       <c r="E46" s="33"/>
       <c r="F46" s="33"/>
       <c r="G46" s="38"/>
-      <c r="H46" s="41"/>
+      <c r="H46" s="40"/>
       <c r="I46" s="35"/>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
@@ -2624,36 +2629,11 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="R12:S12"/>
-    <mergeCell ref="R13:S13"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="R7:S7"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="R9:S9"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="D39:G39"/>
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="Q36:R36"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="D10:H10"/>
@@ -2670,11 +2650,36 @@
     <mergeCell ref="P25:S25"/>
     <mergeCell ref="P28:Q28"/>
     <mergeCell ref="P29:S29"/>
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="D38:G38"/>
-    <mergeCell ref="D39:G39"/>
-    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="R12:S12"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="R20:S20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor print scripts and XML files: update logo image size, enhance data handling, and adjust table column spans for improved layout
</commit_message>
<xml_diff>
--- a/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
+++ b/src/FileCabinet/SuiteScripts/Nkn/xlsx/scv_xlsx_wb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SCV\NAKANO\HOAN_NAKANO\src\FileCabinet\SuiteScripts\Nkn\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548FF733-0829-4D61-A634-96E9730F7893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50F29B47-9F61-4875-8AFB-479F1596DD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FBFDA3B2-B482-4DA1-B36E-083EA194CE53}"/>
   </bookViews>
@@ -366,7 +366,7 @@
     <t>{pIndirectExpensesPer}%</t>
   </si>
   <si>
-    <t xml:space="preserve"> NAKANO SINGAPORE </t>
+    <t xml:space="preserve"> {pSubName}</t>
   </si>
 </sst>
 </file>
@@ -887,12 +887,99 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -909,93 +996,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1335,21 +1335,21 @@
       <c r="A1" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="66" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
       <c r="F1" s="13"/>
-      <c r="G1" s="50" t="s">
+      <c r="G1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
       <c r="M1" s="13"/>
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
@@ -1387,13 +1387,13 @@
       <c r="C3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="64" t="s">
+      <c r="D3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
       <c r="I3" s="10">
         <v>1</v>
       </c>
@@ -1409,10 +1409,10 @@
         <v>101</v>
       </c>
       <c r="O3" s="2"/>
-      <c r="P3" s="51" t="s">
+      <c r="P3" s="64" t="s">
         <v>86</v>
       </c>
-      <c r="Q3" s="51"/>
+      <c r="Q3" s="64"/>
       <c r="R3" s="22"/>
       <c r="S3" s="20"/>
     </row>
@@ -1445,13 +1445,13 @@
       <c r="C5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="69"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
       <c r="I5" s="10">
         <v>2</v>
       </c>
@@ -1467,10 +1467,10 @@
         <v>101</v>
       </c>
       <c r="O5" s="2"/>
-      <c r="P5" s="52" t="s">
+      <c r="P5" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="Q5" s="52"/>
+      <c r="Q5" s="68"/>
       <c r="R5" s="23"/>
       <c r="S5" s="20"/>
     </row>
@@ -1519,14 +1519,14 @@
         <v>101</v>
       </c>
       <c r="O7" s="2"/>
-      <c r="P7" s="51" t="s">
+      <c r="P7" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="Q7" s="51"/>
-      <c r="R7" s="55" t="s">
+      <c r="Q7" s="64"/>
+      <c r="R7" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="S7" s="56"/>
+      <c r="S7" s="70"/>
     </row>
     <row r="8" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
@@ -1550,14 +1550,14 @@
         <v>101</v>
       </c>
       <c r="O8" s="2"/>
-      <c r="P8" s="62" t="s">
+      <c r="P8" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="Q8" s="62"/>
-      <c r="R8" s="57" t="s">
+      <c r="Q8" s="65"/>
+      <c r="R8" s="71" t="s">
         <v>105</v>
       </c>
-      <c r="S8" s="58"/>
+      <c r="S8" s="72"/>
     </row>
     <row r="9" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
@@ -1581,14 +1581,14 @@
         <v>101</v>
       </c>
       <c r="O9" s="2"/>
-      <c r="P9" s="59" t="s">
+      <c r="P9" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="Q9" s="59"/>
-      <c r="R9" s="42" t="s">
+      <c r="Q9" s="55"/>
+      <c r="R9" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="S9" s="43"/>
+      <c r="S9" s="59"/>
     </row>
     <row r="10" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1598,13 +1598,13 @@
       <c r="C10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="64" t="s">
+      <c r="D10" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64"/>
-      <c r="H10" s="64"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -1612,8 +1612,8 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="63"/>
-      <c r="Q10" s="63"/>
+      <c r="P10" s="56"/>
+      <c r="Q10" s="56"/>
       <c r="R10" s="2"/>
       <c r="S10" s="18"/>
     </row>
@@ -1622,10 +1622,10 @@
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="53"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
       <c r="I11" s="10">
         <v>4</v>
       </c>
@@ -1639,10 +1639,10 @@
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="53"/>
-      <c r="Q11" s="53"/>
-      <c r="R11" s="53"/>
-      <c r="S11" s="54"/>
+      <c r="P11" s="47"/>
+      <c r="Q11" s="47"/>
+      <c r="R11" s="47"/>
+      <c r="S11" s="50"/>
     </row>
     <row r="12" spans="1:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
@@ -1664,14 +1664,14 @@
         <v>101</v>
       </c>
       <c r="O12" s="2"/>
-      <c r="P12" s="59" t="s">
+      <c r="P12" s="55" t="s">
         <v>91</v>
       </c>
-      <c r="Q12" s="59"/>
-      <c r="R12" s="42" t="s">
+      <c r="Q12" s="55"/>
+      <c r="R12" s="58" t="s">
         <v>107</v>
       </c>
-      <c r="S12" s="43"/>
+      <c r="S12" s="59"/>
     </row>
     <row r="13" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
@@ -1693,14 +1693,14 @@
         <v>101</v>
       </c>
       <c r="O13" s="2"/>
-      <c r="P13" s="60" t="s">
+      <c r="P13" s="62" t="s">
         <v>92</v>
       </c>
-      <c r="Q13" s="60"/>
-      <c r="R13" s="44" t="s">
+      <c r="Q13" s="62"/>
+      <c r="R13" s="73" t="s">
         <v>108</v>
       </c>
-      <c r="S13" s="45"/>
+      <c r="S13" s="74"/>
     </row>
     <row r="14" spans="1:19" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
@@ -1731,13 +1731,13 @@
       <c r="C15" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="64" t="s">
+      <c r="D15" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="48"/>
       <c r="I15" s="10">
         <v>5</v>
       </c>
@@ -1785,12 +1785,12 @@
       <c r="C17" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="64" t="s">
+      <c r="D17" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="E17" s="64"/>
-      <c r="F17" s="64"/>
-      <c r="G17" s="64"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
       <c r="H17" s="27" t="s">
         <v>12</v>
       </c>
@@ -1807,14 +1807,14 @@
       <c r="O17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P17" s="61" t="s">
+      <c r="P17" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="Q17" s="61"/>
-      <c r="R17" s="46" t="s">
+      <c r="Q17" s="63"/>
+      <c r="R17" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="S17" s="47"/>
+      <c r="S17" s="76"/>
     </row>
     <row r="18" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
@@ -1838,25 +1838,25 @@
       <c r="O18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P18" s="66" t="s">
+      <c r="P18" s="53" t="s">
         <v>94</v>
       </c>
-      <c r="Q18" s="66"/>
-      <c r="R18" s="48" t="s">
+      <c r="Q18" s="53"/>
+      <c r="R18" s="77" t="s">
         <v>49</v>
       </c>
-      <c r="S18" s="49"/>
+      <c r="S18" s="78"/>
     </row>
     <row r="19" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="64" t="s">
+      <c r="D19" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="64"/>
-      <c r="F19" s="64"/>
-      <c r="G19" s="64"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
       <c r="H19" s="27" t="s">
         <v>13</v>
       </c>
@@ -1896,25 +1896,25 @@
       <c r="O20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="P20" s="42" t="s">
+      <c r="P20" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="46" t="s">
+      <c r="Q20" s="58"/>
+      <c r="R20" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="S20" s="47"/>
+      <c r="S20" s="76"/>
     </row>
     <row r="21" spans="1:19" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="64" t="s">
+      <c r="D21" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
       <c r="H21" s="27" t="s">
         <v>14</v>
       </c>
@@ -1961,12 +1961,12 @@
       <c r="A23" s="3"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="64" t="s">
+      <c r="D23" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="64"/>
-      <c r="F23" s="64"/>
-      <c r="G23" s="64"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
       <c r="H23" s="28" t="s">
         <v>15</v>
       </c>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
-      <c r="P23" s="67" t="s">
+      <c r="P23" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="Q23" s="67"/>
-      <c r="R23" s="67"/>
-      <c r="S23" s="68"/>
+      <c r="Q23" s="60"/>
+      <c r="R23" s="60"/>
+      <c r="S23" s="61"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
@@ -2008,23 +2008,23 @@
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
-      <c r="P24" s="66" t="s">
+      <c r="P24" s="53" t="s">
         <v>97</v>
       </c>
-      <c r="Q24" s="66"/>
-      <c r="R24" s="66"/>
-      <c r="S24" s="72"/>
+      <c r="Q24" s="53"/>
+      <c r="R24" s="53"/>
+      <c r="S24" s="54"/>
     </row>
     <row r="25" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-      <c r="D25" s="64" t="s">
+      <c r="D25" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="64"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
       <c r="H25" s="27" t="s">
         <v>16</v>
       </c>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
-      <c r="P25" s="66" t="s">
+      <c r="P25" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="Q25" s="66"/>
-      <c r="R25" s="66"/>
-      <c r="S25" s="72"/>
+      <c r="Q25" s="53"/>
+      <c r="R25" s="53"/>
+      <c r="S25" s="54"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
@@ -2071,12 +2071,12 @@
       <c r="A27" s="3"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="64" t="s">
+      <c r="D27" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
       <c r="H27" s="27" t="s">
         <v>17</v>
       </c>
@@ -2118,14 +2118,14 @@
         <v>101</v>
       </c>
       <c r="O28" s="2"/>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="Q28" s="59"/>
-      <c r="R28" s="42" t="s">
+      <c r="Q28" s="55"/>
+      <c r="R28" s="58" t="s">
         <v>109</v>
       </c>
-      <c r="S28" s="43"/>
+      <c r="S28" s="59"/>
     </row>
     <row r="29" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -2135,12 +2135,12 @@
       <c r="C29" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D29" s="65" t="s">
+      <c r="D29" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="65"/>
-      <c r="F29" s="65"/>
-      <c r="G29" s="65"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
       <c r="H29" s="27"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -2149,10 +2149,10 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
-      <c r="P29" s="63"/>
-      <c r="Q29" s="63"/>
-      <c r="R29" s="63"/>
-      <c r="S29" s="73"/>
+      <c r="P29" s="56"/>
+      <c r="Q29" s="56"/>
+      <c r="R29" s="56"/>
+      <c r="S29" s="57"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -2162,11 +2162,11 @@
       <c r="C30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D30" s="70" t="s">
+      <c r="D30" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
       <c r="G30" s="29" t="s">
         <v>58</v>
       </c>
@@ -2178,10 +2178,10 @@
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
-      <c r="P30" s="53"/>
-      <c r="Q30" s="53"/>
-      <c r="R30" s="53"/>
-      <c r="S30" s="54"/>
+      <c r="P30" s="47"/>
+      <c r="Q30" s="47"/>
+      <c r="R30" s="47"/>
+      <c r="S30" s="50"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -2191,11 +2191,11 @@
       <c r="C31" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D31" s="65" t="s">
+      <c r="D31" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="65"/>
-      <c r="F31" s="65"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="51"/>
       <c r="G31" s="27" t="s">
         <v>60</v>
       </c>
@@ -2220,12 +2220,12 @@
       <c r="C32" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D32" s="71" t="s">
+      <c r="D32" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="E32" s="71"/>
-      <c r="F32" s="71"/>
-      <c r="G32" s="71"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="52"/>
       <c r="H32" s="25"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -2247,11 +2247,11 @@
       <c r="C33" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D33" s="71" t="s">
+      <c r="D33" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="E33" s="71"/>
-      <c r="F33" s="71"/>
+      <c r="E33" s="52"/>
+      <c r="F33" s="52"/>
       <c r="G33" s="25" t="s">
         <v>62</v>
       </c>
@@ -2320,12 +2320,12 @@
       <c r="C36" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D36" s="74" t="s">
+      <c r="D36" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="E36" s="74"/>
-      <c r="F36" s="74"/>
-      <c r="G36" s="74"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="43"/>
       <c r="H36" s="4"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -2335,8 +2335,8 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
-      <c r="Q36" s="53"/>
-      <c r="R36" s="53"/>
+      <c r="Q36" s="47"/>
+      <c r="R36" s="47"/>
       <c r="S36" s="18"/>
     </row>
     <row r="37" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2347,12 +2347,12 @@
       <c r="C37" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D37" s="75" t="s">
+      <c r="D37" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="E37" s="75"/>
-      <c r="F37" s="75"/>
-      <c r="G37" s="75"/>
+      <c r="E37" s="44"/>
+      <c r="F37" s="44"/>
+      <c r="G37" s="44"/>
       <c r="H37" s="4"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -2374,12 +2374,12 @@
       <c r="C38" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D38" s="75" t="s">
+      <c r="D38" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="75"/>
+      <c r="E38" s="44"/>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
       <c r="H38" s="4" t="s">
         <v>24</v>
       </c>
@@ -2403,12 +2403,12 @@
       <c r="C39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D39" s="76" t="s">
+      <c r="D39" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="45"/>
+      <c r="G39" s="45"/>
       <c r="H39" s="4" t="s">
         <v>24</v>
       </c>
@@ -2432,12 +2432,12 @@
       <c r="C40" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D40" s="70" t="s">
+      <c r="D40" s="46" t="s">
         <v>79</v>
       </c>
-      <c r="E40" s="70"/>
-      <c r="F40" s="70"/>
-      <c r="G40" s="70"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="46"/>
       <c r="H40" s="4" t="s">
         <v>24</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>65</v>
       </c>
       <c r="F45" s="2"/>
-      <c r="G45" s="77" t="s">
+      <c r="G45" s="42" t="s">
         <v>85</v>
       </c>
       <c r="H45" s="10" t="s">
@@ -2629,11 +2629,36 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="D38:G38"/>
-    <mergeCell ref="D39:G39"/>
-    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="R12:S12"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="D23:G23"/>
     <mergeCell ref="Q36:R36"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="D10:H10"/>
@@ -2650,36 +2675,11 @@
     <mergeCell ref="P25:S25"/>
     <mergeCell ref="P28:Q28"/>
     <mergeCell ref="P29:S29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="R7:S7"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="R9:S9"/>
-    <mergeCell ref="R12:S12"/>
-    <mergeCell ref="R13:S13"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="D39:G39"/>
+    <mergeCell ref="D40:G40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>